<commit_message>
Add Use (ON/OFF) column and multi-port function dropdowns
- RC40_Pinmap.xlsx: new H column 'Use' (ON/OFF dropdown, default ON) and
  C column 'Type' dropdowns for 36 multi-port pins, built from Description
- Use=OFF pins are generated under Unused/HwInp|HwOutp/<class> and excluded
  from the BSW integration snippets (cfg.unusedGroup)
- Multi-port pins: direction follows the selected function (e.g. K62 Digital
  -> HwInp/Dig, Analog output -> HwOutp/AbsltU); warning if the selected Type
  is not listed in the Description
- New CurrentSignal type -> HwInp/AnI (i_uA_u16, 0..25000 uA), with guide and
  snippet support
- tools/add_pinmap_dropdowns.py (stdlib only) rebuilds the dropdowns
- README updated
</commit_message>
<xml_diff>
--- a/RC40_Pinmap.xlsx
+++ b/RC40_Pinmap.xlsx
@@ -1438,7 +1438,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C38D0752-6C4A-40D7-A9B9-7CD12FA937BE}">
-  <dimension ref="B1:G162"/>
+  <dimension ref="B1:H162"/>
   <sheetFormatPr defaultRowHeight="16.5"/>
   <cols>
     <col min="2" max="2" width="8.75" bestFit="1" customWidth="1"/>
@@ -1446,6 +1446,7 @@
     <col min="5" max="5" width="48.5" customWidth="1"/>
     <col min="6" max="6" width="16.375" style="17" customWidth="1"/>
     <col min="7" max="7" width="22.375" style="17" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:7" ht="20.25">
@@ -1458,7 +1459,7 @@
       <c r="F1" s="22"/>
       <c r="G1" s="23"/>
     </row>
-    <row r="2" spans="2:7" ht="33">
+    <row r="2" spans="2:8" ht="33">
       <c r="B2" s="13" t="s">
         <v>130</v>
       </c>
@@ -1477,8 +1478,13 @@
       <c r="G2" s="13" t="s">
         <v>227</v>
       </c>
-    </row>
-    <row r="3" spans="2:7" ht="33">
+      <c r="H2" s="13" t="inlineStr">
+        <is>
+          <t>Use</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" spans="2:8" ht="33">
       <c r="B3" s="3" t="s">
         <v>0</v>
       </c>
@@ -1493,8 +1499,13 @@
       </c>
       <c r="F3" s="3"/>
       <c r="G3" s="15"/>
-    </row>
-    <row r="4" spans="2:7" ht="33">
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" spans="2:8" ht="33">
       <c r="B4" s="3" t="s">
         <v>1</v>
       </c>
@@ -1509,8 +1520,13 @@
       </c>
       <c r="F4" s="3"/>
       <c r="G4" s="15"/>
-    </row>
-    <row r="5" spans="2:7" ht="33">
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" spans="2:8" ht="33">
       <c r="B5" s="3" t="s">
         <v>2</v>
       </c>
@@ -1525,8 +1541,13 @@
       </c>
       <c r="F5" s="3"/>
       <c r="G5" s="15"/>
-    </row>
-    <row r="6" spans="2:7" ht="33">
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" spans="2:8" ht="33">
       <c r="B6" s="3" t="s">
         <v>3</v>
       </c>
@@ -1541,8 +1562,13 @@
       </c>
       <c r="F6" s="3"/>
       <c r="G6" s="15"/>
-    </row>
-    <row r="7" spans="2:7" ht="33">
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" spans="2:8" ht="33">
       <c r="B7" s="3" t="s">
         <v>4</v>
       </c>
@@ -1557,8 +1583,13 @@
       </c>
       <c r="F7" s="3"/>
       <c r="G7" s="15"/>
-    </row>
-    <row r="8" spans="2:7" ht="33">
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" spans="2:8" ht="33">
       <c r="B8" s="3" t="s">
         <v>5</v>
       </c>
@@ -1573,8 +1604,13 @@
       </c>
       <c r="F8" s="3"/>
       <c r="G8" s="15"/>
-    </row>
-    <row r="9" spans="2:7" ht="33">
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" spans="2:8" ht="33">
       <c r="B9" s="3" t="s">
         <v>6</v>
       </c>
@@ -1589,8 +1625,13 @@
       </c>
       <c r="F9" s="3"/>
       <c r="G9" s="15"/>
-    </row>
-    <row r="10" spans="2:7" ht="33">
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" spans="2:8" ht="33">
       <c r="B10" s="3" t="s">
         <v>7</v>
       </c>
@@ -1605,8 +1646,13 @@
       </c>
       <c r="F10" s="3"/>
       <c r="G10" s="15"/>
-    </row>
-    <row r="11" spans="2:7" ht="33">
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" spans="2:8" ht="33">
       <c r="B11" s="3" t="s">
         <v>8</v>
       </c>
@@ -1621,8 +1667,13 @@
       </c>
       <c r="F11" s="3"/>
       <c r="G11" s="15"/>
-    </row>
-    <row r="12" spans="2:7" ht="33">
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" spans="2:8" ht="33">
       <c r="B12" s="3" t="s">
         <v>9</v>
       </c>
@@ -1637,8 +1688,13 @@
       </c>
       <c r="F12" s="3"/>
       <c r="G12" s="15"/>
-    </row>
-    <row r="13" spans="2:7" ht="33">
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" spans="2:8" ht="33">
       <c r="B13" s="3" t="s">
         <v>10</v>
       </c>
@@ -1653,8 +1709,13 @@
       </c>
       <c r="F13" s="3"/>
       <c r="G13" s="15"/>
-    </row>
-    <row r="14" spans="2:7" ht="49.5">
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" spans="2:8" ht="49.5">
       <c r="B14" s="3" t="s">
         <v>11</v>
       </c>
@@ -1669,8 +1730,13 @@
       </c>
       <c r="F14" s="3"/>
       <c r="G14" s="15"/>
-    </row>
-    <row r="15" spans="2:7">
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" spans="2:8">
       <c r="B15" s="3" t="s">
         <v>12</v>
       </c>
@@ -1685,8 +1751,13 @@
       </c>
       <c r="F15" s="3"/>
       <c r="G15" s="15"/>
-    </row>
-    <row r="16" spans="2:7">
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" spans="2:8">
       <c r="B16" s="3" t="s">
         <v>13</v>
       </c>
@@ -1701,8 +1772,13 @@
       </c>
       <c r="F16" s="3"/>
       <c r="G16" s="15"/>
-    </row>
-    <row r="17" spans="2:7" ht="33">
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" spans="2:8" ht="33">
       <c r="B17" s="3" t="s">
         <v>14</v>
       </c>
@@ -1717,8 +1793,13 @@
       </c>
       <c r="F17" s="3"/>
       <c r="G17" s="15"/>
-    </row>
-    <row r="18" spans="2:7" ht="33">
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" spans="2:8" ht="33">
       <c r="B18" s="3" t="s">
         <v>15</v>
       </c>
@@ -1733,8 +1814,13 @@
       </c>
       <c r="F18" s="3"/>
       <c r="G18" s="15"/>
-    </row>
-    <row r="19" spans="2:7" ht="33">
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" spans="2:8" ht="33">
       <c r="B19" s="3" t="s">
         <v>16</v>
       </c>
@@ -1749,8 +1835,13 @@
       </c>
       <c r="F19" s="3"/>
       <c r="G19" s="15"/>
-    </row>
-    <row r="20" spans="2:7" ht="33">
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" spans="2:8" ht="33">
       <c r="B20" s="3" t="s">
         <v>17</v>
       </c>
@@ -1765,8 +1856,13 @@
       </c>
       <c r="F20" s="3"/>
       <c r="G20" s="15"/>
-    </row>
-    <row r="21" spans="2:7" ht="33">
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" spans="2:8" ht="33">
       <c r="B21" s="3" t="s">
         <v>18</v>
       </c>
@@ -1781,8 +1877,13 @@
       </c>
       <c r="F21" s="3"/>
       <c r="G21" s="15"/>
-    </row>
-    <row r="22" spans="2:7">
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" spans="2:8">
       <c r="B22" s="3" t="s">
         <v>19</v>
       </c>
@@ -1797,8 +1898,13 @@
       </c>
       <c r="F22" s="3"/>
       <c r="G22" s="15"/>
-    </row>
-    <row r="23" spans="2:7">
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" spans="2:8">
       <c r="B23" s="3" t="s">
         <v>20</v>
       </c>
@@ -1813,8 +1919,13 @@
       </c>
       <c r="F23" s="3"/>
       <c r="G23" s="15"/>
-    </row>
-    <row r="24" spans="2:7">
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" spans="2:8">
       <c r="B24" s="3" t="s">
         <v>21</v>
       </c>
@@ -1829,8 +1940,13 @@
       </c>
       <c r="F24" s="3"/>
       <c r="G24" s="15"/>
-    </row>
-    <row r="25" spans="2:7">
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" spans="2:8">
       <c r="B25" s="3" t="s">
         <v>22</v>
       </c>
@@ -1845,8 +1961,13 @@
       </c>
       <c r="F25" s="3"/>
       <c r="G25" s="15"/>
-    </row>
-    <row r="26" spans="2:7">
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" spans="2:8">
       <c r="B26" s="3" t="s">
         <v>23</v>
       </c>
@@ -1861,8 +1982,13 @@
       </c>
       <c r="F26" s="3"/>
       <c r="G26" s="15"/>
-    </row>
-    <row r="27" spans="2:7">
+      <c r="H26" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" spans="2:8">
       <c r="B27" s="3" t="s">
         <v>24</v>
       </c>
@@ -1877,8 +2003,13 @@
       </c>
       <c r="F27" s="3"/>
       <c r="G27" s="15"/>
-    </row>
-    <row r="28" spans="2:7">
+      <c r="H27" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" spans="2:8">
       <c r="B28" s="3" t="s">
         <v>25</v>
       </c>
@@ -1893,8 +2024,13 @@
       </c>
       <c r="F28" s="3"/>
       <c r="G28" s="15"/>
-    </row>
-    <row r="29" spans="2:7">
+      <c r="H28" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" spans="2:8">
       <c r="B29" s="3" t="s">
         <v>26</v>
       </c>
@@ -1909,8 +2045,13 @@
       </c>
       <c r="F29" s="3"/>
       <c r="G29" s="15"/>
-    </row>
-    <row r="30" spans="2:7">
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" spans="2:8">
       <c r="B30" s="3" t="s">
         <v>27</v>
       </c>
@@ -1925,8 +2066,13 @@
       </c>
       <c r="F30" s="3"/>
       <c r="G30" s="15"/>
-    </row>
-    <row r="31" spans="2:7" ht="33">
+      <c r="H30" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" spans="2:8" ht="33">
       <c r="B31" s="3" t="s">
         <v>28</v>
       </c>
@@ -1941,8 +2087,13 @@
       </c>
       <c r="F31" s="3"/>
       <c r="G31" s="15"/>
-    </row>
-    <row r="32" spans="2:7" ht="33">
+      <c r="H31" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" spans="2:8" ht="33">
       <c r="B32" s="3" t="s">
         <v>29</v>
       </c>
@@ -1957,8 +2108,13 @@
       </c>
       <c r="F32" s="3"/>
       <c r="G32" s="15"/>
-    </row>
-    <row r="33" spans="2:7" ht="33">
+      <c r="H32" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" spans="2:8" ht="33">
       <c r="B33" s="3" t="s">
         <v>30</v>
       </c>
@@ -1973,8 +2129,13 @@
       </c>
       <c r="F33" s="3"/>
       <c r="G33" s="15"/>
-    </row>
-    <row r="34" spans="2:7" ht="33">
+      <c r="H33" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" spans="2:8" ht="33">
       <c r="B34" s="3" t="s">
         <v>31</v>
       </c>
@@ -1989,8 +2150,13 @@
       </c>
       <c r="F34" s="3"/>
       <c r="G34" s="15"/>
-    </row>
-    <row r="35" spans="2:7" ht="33">
+      <c r="H34" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" spans="2:8" ht="33">
       <c r="B35" s="3" t="s">
         <v>32</v>
       </c>
@@ -2005,8 +2171,13 @@
       </c>
       <c r="F35" s="3"/>
       <c r="G35" s="15"/>
-    </row>
-    <row r="36" spans="2:7">
+      <c r="H35" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" spans="2:8">
       <c r="B36" s="3" t="s">
         <v>33</v>
       </c>
@@ -2021,8 +2192,13 @@
       </c>
       <c r="F36" s="3"/>
       <c r="G36" s="15"/>
-    </row>
-    <row r="37" spans="2:7">
+      <c r="H36" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" spans="2:8">
       <c r="B37" s="3" t="s">
         <v>34</v>
       </c>
@@ -2037,8 +2213,13 @@
       </c>
       <c r="F37" s="3"/>
       <c r="G37" s="15"/>
-    </row>
-    <row r="38" spans="2:7">
+      <c r="H37" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" spans="2:8">
       <c r="B38" s="3" t="s">
         <v>35</v>
       </c>
@@ -2053,8 +2234,13 @@
       </c>
       <c r="F38" s="3"/>
       <c r="G38" s="15"/>
-    </row>
-    <row r="39" spans="2:7">
+      <c r="H38" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" spans="2:8">
       <c r="B39" s="3" t="s">
         <v>36</v>
       </c>
@@ -2069,8 +2255,13 @@
       </c>
       <c r="F39" s="3"/>
       <c r="G39" s="15"/>
-    </row>
-    <row r="40" spans="2:7">
+      <c r="H39" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" spans="2:8">
       <c r="B40" s="3" t="s">
         <v>37</v>
       </c>
@@ -2085,8 +2276,13 @@
       </c>
       <c r="F40" s="3"/>
       <c r="G40" s="15"/>
-    </row>
-    <row r="41" spans="2:7">
+      <c r="H40" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" spans="2:8">
       <c r="B41" s="3" t="s">
         <v>38</v>
       </c>
@@ -2101,8 +2297,13 @@
       </c>
       <c r="F41" s="3"/>
       <c r="G41" s="15"/>
-    </row>
-    <row r="42" spans="2:7">
+      <c r="H41" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" spans="2:8">
       <c r="B42" s="3" t="s">
         <v>39</v>
       </c>
@@ -2117,8 +2318,13 @@
       </c>
       <c r="F42" s="3"/>
       <c r="G42" s="15"/>
-    </row>
-    <row r="43" spans="2:7">
+      <c r="H42" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" spans="2:8">
       <c r="B43" s="3" t="s">
         <v>40</v>
       </c>
@@ -2133,8 +2339,13 @@
       </c>
       <c r="F43" s="3"/>
       <c r="G43" s="15"/>
-    </row>
-    <row r="44" spans="2:7">
+      <c r="H43" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" spans="2:8">
       <c r="B44" s="3" t="s">
         <v>41</v>
       </c>
@@ -2147,8 +2358,13 @@
       <c r="E44" s="1"/>
       <c r="F44" s="3"/>
       <c r="G44" s="15"/>
-    </row>
-    <row r="45" spans="2:7" ht="33">
+      <c r="H44" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" spans="2:8" ht="33">
       <c r="B45" s="3" t="s">
         <v>42</v>
       </c>
@@ -2163,8 +2379,13 @@
       </c>
       <c r="F45" s="3"/>
       <c r="G45" s="15"/>
-    </row>
-    <row r="46" spans="2:7" ht="33">
+      <c r="H45" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" spans="2:8" ht="33">
       <c r="B46" s="3" t="s">
         <v>43</v>
       </c>
@@ -2179,8 +2400,13 @@
       </c>
       <c r="F46" s="3"/>
       <c r="G46" s="15"/>
-    </row>
-    <row r="47" spans="2:7" ht="33">
+      <c r="H46" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" spans="2:8" ht="33">
       <c r="B47" s="3" t="s">
         <v>44</v>
       </c>
@@ -2195,8 +2421,13 @@
       </c>
       <c r="F47" s="3"/>
       <c r="G47" s="15"/>
-    </row>
-    <row r="48" spans="2:7" ht="33">
+      <c r="H47" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" spans="2:8" ht="33">
       <c r="B48" s="3" t="s">
         <v>45</v>
       </c>
@@ -2211,8 +2442,13 @@
       </c>
       <c r="F48" s="3"/>
       <c r="G48" s="15"/>
-    </row>
-    <row r="49" spans="2:7" ht="33">
+      <c r="H48" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" spans="2:8" ht="33">
       <c r="B49" s="3" t="s">
         <v>46</v>
       </c>
@@ -2227,8 +2463,13 @@
       </c>
       <c r="F49" s="3"/>
       <c r="G49" s="15"/>
-    </row>
-    <row r="50" spans="2:7" ht="33">
+      <c r="H49" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" spans="2:8" ht="33">
       <c r="B50" s="3" t="s">
         <v>47</v>
       </c>
@@ -2243,8 +2484,13 @@
       </c>
       <c r="F50" s="3"/>
       <c r="G50" s="15"/>
-    </row>
-    <row r="51" spans="2:7" ht="33">
+      <c r="H50" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" spans="2:8" ht="33">
       <c r="B51" s="3" t="s">
         <v>48</v>
       </c>
@@ -2259,8 +2505,13 @@
       </c>
       <c r="F51" s="3"/>
       <c r="G51" s="15"/>
-    </row>
-    <row r="52" spans="2:7" ht="33">
+      <c r="H51" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" spans="2:8" ht="33">
       <c r="B52" s="3" t="s">
         <v>49</v>
       </c>
@@ -2275,8 +2526,13 @@
       </c>
       <c r="F52" s="3"/>
       <c r="G52" s="15"/>
-    </row>
-    <row r="53" spans="2:7" ht="33">
+      <c r="H52" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" spans="2:8" ht="33">
       <c r="B53" s="3" t="s">
         <v>50</v>
       </c>
@@ -2291,8 +2547,13 @@
       </c>
       <c r="F53" s="3"/>
       <c r="G53" s="15"/>
-    </row>
-    <row r="54" spans="2:7" ht="33">
+      <c r="H53" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" spans="2:8" ht="33">
       <c r="B54" s="3" t="s">
         <v>51</v>
       </c>
@@ -2307,8 +2568,13 @@
       </c>
       <c r="F54" s="3"/>
       <c r="G54" s="15"/>
-    </row>
-    <row r="55" spans="2:7" ht="33">
+      <c r="H54" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" spans="2:8" ht="33">
       <c r="B55" s="3" t="s">
         <v>52</v>
       </c>
@@ -2323,8 +2589,13 @@
       </c>
       <c r="F55" s="3"/>
       <c r="G55" s="15"/>
-    </row>
-    <row r="56" spans="2:7">
+      <c r="H55" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" spans="2:8">
       <c r="B56" s="3" t="s">
         <v>53</v>
       </c>
@@ -2339,8 +2610,13 @@
       </c>
       <c r="F56" s="3"/>
       <c r="G56" s="15"/>
-    </row>
-    <row r="57" spans="2:7" ht="33">
+      <c r="H56" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" spans="2:8" ht="33">
       <c r="B57" s="3" t="s">
         <v>54</v>
       </c>
@@ -2355,8 +2631,13 @@
       </c>
       <c r="F57" s="3"/>
       <c r="G57" s="15"/>
-    </row>
-    <row r="58" spans="2:7">
+      <c r="H57" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" spans="2:8">
       <c r="B58" s="3" t="s">
         <v>55</v>
       </c>
@@ -2369,8 +2650,13 @@
       <c r="E58" s="1"/>
       <c r="F58" s="3"/>
       <c r="G58" s="15"/>
-    </row>
-    <row r="59" spans="2:7">
+      <c r="H58" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" spans="2:8">
       <c r="B59" s="3" t="s">
         <v>56</v>
       </c>
@@ -2385,8 +2671,13 @@
       </c>
       <c r="F59" s="3"/>
       <c r="G59" s="15"/>
-    </row>
-    <row r="60" spans="2:7" ht="33">
+      <c r="H59" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" spans="2:8" ht="33">
       <c r="B60" s="3" t="s">
         <v>57</v>
       </c>
@@ -2401,8 +2692,13 @@
       </c>
       <c r="F60" s="3"/>
       <c r="G60" s="15"/>
-    </row>
-    <row r="61" spans="2:7" ht="33">
+      <c r="H60" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" spans="2:8" ht="33">
       <c r="B61" s="3" t="s">
         <v>58</v>
       </c>
@@ -2417,8 +2713,13 @@
       </c>
       <c r="F61" s="3"/>
       <c r="G61" s="15"/>
-    </row>
-    <row r="62" spans="2:7" ht="33">
+      <c r="H61" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" spans="2:8" ht="33">
       <c r="B62" s="3" t="s">
         <v>59</v>
       </c>
@@ -2433,8 +2734,13 @@
       </c>
       <c r="F62" s="3"/>
       <c r="G62" s="15"/>
-    </row>
-    <row r="63" spans="2:7">
+      <c r="H62" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" spans="2:8">
       <c r="B63" s="3" t="s">
         <v>60</v>
       </c>
@@ -2449,8 +2755,13 @@
       </c>
       <c r="F63" s="3"/>
       <c r="G63" s="15"/>
-    </row>
-    <row r="64" spans="2:7">
+      <c r="H63" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" spans="2:8">
       <c r="B64" s="3" t="s">
         <v>61</v>
       </c>
@@ -2465,8 +2776,13 @@
       </c>
       <c r="F64" s="3"/>
       <c r="G64" s="15"/>
-    </row>
-    <row r="65" spans="2:7" ht="33">
+      <c r="H64" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" spans="2:8" ht="33">
       <c r="B65" s="3" t="s">
         <v>62</v>
       </c>
@@ -2481,8 +2797,13 @@
       </c>
       <c r="F65" s="3"/>
       <c r="G65" s="15"/>
-    </row>
-    <row r="66" spans="2:7" ht="33">
+      <c r="H65" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" spans="2:8" ht="33">
       <c r="B66" s="3" t="s">
         <v>63</v>
       </c>
@@ -2497,8 +2818,13 @@
       </c>
       <c r="F66" s="3"/>
       <c r="G66" s="15"/>
-    </row>
-    <row r="67" spans="2:7" ht="33">
+      <c r="H66" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" spans="2:8" ht="33">
       <c r="B67" s="3" t="s">
         <v>64</v>
       </c>
@@ -2513,8 +2839,13 @@
       </c>
       <c r="F67" s="3"/>
       <c r="G67" s="15"/>
-    </row>
-    <row r="68" spans="2:7" ht="33">
+      <c r="H67" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" spans="2:8" ht="33">
       <c r="B68" s="3" t="s">
         <v>65</v>
       </c>
@@ -2529,8 +2860,13 @@
       </c>
       <c r="F68" s="3"/>
       <c r="G68" s="15"/>
-    </row>
-    <row r="69" spans="2:7" ht="33">
+      <c r="H68" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" spans="2:8" ht="33">
       <c r="B69" s="3" t="s">
         <v>66</v>
       </c>
@@ -2545,8 +2881,13 @@
       </c>
       <c r="F69" s="3"/>
       <c r="G69" s="15"/>
-    </row>
-    <row r="70" spans="2:7">
+      <c r="H69" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" spans="2:8">
       <c r="B70" s="3" t="s">
         <v>67</v>
       </c>
@@ -2561,8 +2902,13 @@
       </c>
       <c r="F70" s="3"/>
       <c r="G70" s="15"/>
-    </row>
-    <row r="71" spans="2:7">
+      <c r="H70" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" spans="2:8">
       <c r="B71" s="3" t="s">
         <v>68</v>
       </c>
@@ -2577,8 +2923,13 @@
       </c>
       <c r="F71" s="3"/>
       <c r="G71" s="15"/>
-    </row>
-    <row r="72" spans="2:7">
+      <c r="H71" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" spans="2:8">
       <c r="B72" s="3" t="s">
         <v>69</v>
       </c>
@@ -2593,8 +2944,13 @@
       </c>
       <c r="F72" s="3"/>
       <c r="G72" s="15"/>
-    </row>
-    <row r="73" spans="2:7" ht="49.5">
+      <c r="H72" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" spans="2:8" ht="49.5">
       <c r="B73" s="3" t="s">
         <v>70</v>
       </c>
@@ -2609,8 +2965,13 @@
       </c>
       <c r="F73" s="3"/>
       <c r="G73" s="15"/>
-    </row>
-    <row r="74" spans="2:7" ht="33">
+      <c r="H73" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" spans="2:8" ht="33">
       <c r="B74" s="3" t="s">
         <v>71</v>
       </c>
@@ -2625,8 +2986,13 @@
       </c>
       <c r="F74" s="3"/>
       <c r="G74" s="15"/>
-    </row>
-    <row r="75" spans="2:7">
+      <c r="H74" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" spans="2:8">
       <c r="B75" s="3" t="s">
         <v>72</v>
       </c>
@@ -2641,8 +3007,13 @@
       </c>
       <c r="F75" s="3"/>
       <c r="G75" s="15"/>
-    </row>
-    <row r="76" spans="2:7">
+      <c r="H75" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" spans="2:8">
       <c r="B76" s="3" t="s">
         <v>73</v>
       </c>
@@ -2655,8 +3026,13 @@
       <c r="E76" s="1"/>
       <c r="F76" s="3"/>
       <c r="G76" s="15"/>
-    </row>
-    <row r="77" spans="2:7">
+      <c r="H76" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" spans="2:8">
       <c r="B77" s="3" t="s">
         <v>74</v>
       </c>
@@ -2671,8 +3047,13 @@
       </c>
       <c r="F77" s="3"/>
       <c r="G77" s="15"/>
-    </row>
-    <row r="78" spans="2:7">
+      <c r="H77" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" spans="2:8">
       <c r="B78" s="3" t="s">
         <v>75</v>
       </c>
@@ -2687,8 +3068,13 @@
       </c>
       <c r="F78" s="3"/>
       <c r="G78" s="15"/>
-    </row>
-    <row r="79" spans="2:7">
+      <c r="H78" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" spans="2:8">
       <c r="B79" s="3" t="s">
         <v>76</v>
       </c>
@@ -2703,8 +3089,13 @@
       </c>
       <c r="F79" s="3"/>
       <c r="G79" s="15"/>
-    </row>
-    <row r="80" spans="2:7">
+      <c r="H79" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" spans="2:8">
       <c r="B80" s="3" t="s">
         <v>77</v>
       </c>
@@ -2719,8 +3110,13 @@
       </c>
       <c r="F80" s="3"/>
       <c r="G80" s="15"/>
-    </row>
-    <row r="81" spans="2:7">
+      <c r="H80" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" spans="2:8">
       <c r="B81" s="3" t="s">
         <v>78</v>
       </c>
@@ -2735,8 +3131,13 @@
       </c>
       <c r="F81" s="3"/>
       <c r="G81" s="15"/>
-    </row>
-    <row r="82" spans="2:7">
+      <c r="H81" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" spans="2:8">
       <c r="B82" s="3" t="s">
         <v>79</v>
       </c>
@@ -2751,8 +3152,13 @@
       </c>
       <c r="F82" s="3"/>
       <c r="G82" s="15"/>
-    </row>
-    <row r="83" spans="2:7">
+      <c r="H82" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" spans="2:8">
       <c r="B83" s="3" t="s">
         <v>80</v>
       </c>
@@ -2767,8 +3173,13 @@
       </c>
       <c r="F83" s="3"/>
       <c r="G83" s="15"/>
-    </row>
-    <row r="84" spans="2:7">
+      <c r="H83" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" spans="2:8">
       <c r="B84" s="3" t="s">
         <v>81</v>
       </c>
@@ -2781,8 +3192,13 @@
       <c r="E84" s="1"/>
       <c r="F84" s="3"/>
       <c r="G84" s="15"/>
-    </row>
-    <row r="85" spans="2:7">
+      <c r="H84" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" spans="2:8">
       <c r="B85" s="3" t="s">
         <v>82</v>
       </c>
@@ -2797,8 +3213,13 @@
       </c>
       <c r="F85" s="3"/>
       <c r="G85" s="15"/>
-    </row>
-    <row r="86" spans="2:7">
+      <c r="H85" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" spans="2:8">
       <c r="B86" s="3" t="s">
         <v>83</v>
       </c>
@@ -2813,8 +3234,13 @@
       </c>
       <c r="F86" s="3"/>
       <c r="G86" s="15"/>
-    </row>
-    <row r="87" spans="2:7">
+      <c r="H86" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" spans="2:8">
       <c r="B87" s="3" t="s">
         <v>84</v>
       </c>
@@ -2829,8 +3255,13 @@
       </c>
       <c r="F87" s="3"/>
       <c r="G87" s="15"/>
-    </row>
-    <row r="88" spans="2:7">
+      <c r="H87" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" spans="2:8">
       <c r="B88" s="3" t="s">
         <v>85</v>
       </c>
@@ -2845,8 +3276,13 @@
       </c>
       <c r="F88" s="3"/>
       <c r="G88" s="15"/>
-    </row>
-    <row r="89" spans="2:7">
+      <c r="H88" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" spans="2:8">
       <c r="B89" s="3" t="s">
         <v>86</v>
       </c>
@@ -2861,8 +3297,13 @@
       </c>
       <c r="F89" s="3"/>
       <c r="G89" s="15"/>
-    </row>
-    <row r="90" spans="2:7">
+      <c r="H89" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" spans="2:8">
       <c r="B90" s="3" t="s">
         <v>87</v>
       </c>
@@ -2877,8 +3318,13 @@
       </c>
       <c r="F90" s="3"/>
       <c r="G90" s="15"/>
-    </row>
-    <row r="91" spans="2:7">
+      <c r="H90" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" spans="2:8">
       <c r="B91" s="3" t="s">
         <v>88</v>
       </c>
@@ -2893,8 +3339,13 @@
       </c>
       <c r="F91" s="3"/>
       <c r="G91" s="15"/>
-    </row>
-    <row r="92" spans="2:7">
+      <c r="H91" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" spans="2:8">
       <c r="B92" s="3" t="s">
         <v>89</v>
       </c>
@@ -2909,8 +3360,13 @@
       </c>
       <c r="F92" s="3"/>
       <c r="G92" s="15"/>
-    </row>
-    <row r="93" spans="2:7" ht="33">
+      <c r="H92" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" spans="2:8" ht="33">
       <c r="B93" s="3" t="s">
         <v>90</v>
       </c>
@@ -2925,8 +3381,13 @@
       </c>
       <c r="F93" s="3"/>
       <c r="G93" s="15"/>
-    </row>
-    <row r="94" spans="2:7">
+      <c r="H93" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" spans="2:8">
       <c r="B94" s="3" t="s">
         <v>91</v>
       </c>
@@ -2941,8 +3402,13 @@
       </c>
       <c r="F94" s="3"/>
       <c r="G94" s="15"/>
-    </row>
-    <row r="95" spans="2:7">
+      <c r="H94" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" spans="2:8">
       <c r="B95" s="3" t="s">
         <v>92</v>
       </c>
@@ -2957,8 +3423,13 @@
       </c>
       <c r="F95" s="3"/>
       <c r="G95" s="15"/>
-    </row>
-    <row r="96" spans="2:7">
+      <c r="H95" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" spans="2:8">
       <c r="B96" s="3" t="s">
         <v>93</v>
       </c>
@@ -2973,8 +3444,13 @@
       </c>
       <c r="F96" s="3"/>
       <c r="G96" s="15"/>
-    </row>
-    <row r="97" spans="2:7">
+      <c r="H96" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" spans="2:8">
       <c r="B97" s="3" t="s">
         <v>94</v>
       </c>
@@ -2987,8 +3463,13 @@
       <c r="E97" s="1"/>
       <c r="F97" s="3"/>
       <c r="G97" s="15"/>
-    </row>
-    <row r="98" spans="2:7">
+      <c r="H97" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" spans="2:8">
       <c r="B98" s="3" t="s">
         <v>95</v>
       </c>
@@ -3003,8 +3484,13 @@
       </c>
       <c r="F98" s="3"/>
       <c r="G98" s="15"/>
-    </row>
-    <row r="99" spans="2:7">
+      <c r="H98" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="99" spans="2:8">
       <c r="B99" s="3" t="s">
         <v>96</v>
       </c>
@@ -3017,8 +3503,13 @@
       <c r="E99" s="1"/>
       <c r="F99" s="3"/>
       <c r="G99" s="15"/>
-    </row>
-    <row r="100" spans="2:7">
+      <c r="H99" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" spans="2:8">
       <c r="B100" s="3" t="s">
         <v>97</v>
       </c>
@@ -3033,8 +3524,13 @@
       </c>
       <c r="F100" s="3"/>
       <c r="G100" s="15"/>
-    </row>
-    <row r="101" spans="2:7">
+      <c r="H100" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" spans="2:8">
       <c r="B101" s="3" t="s">
         <v>98</v>
       </c>
@@ -3049,8 +3545,13 @@
       </c>
       <c r="F101" s="3"/>
       <c r="G101" s="15"/>
-    </row>
-    <row r="102" spans="2:7">
+      <c r="H101" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" spans="2:8">
       <c r="B102" s="3" t="s">
         <v>99</v>
       </c>
@@ -3065,8 +3566,13 @@
       </c>
       <c r="F102" s="3"/>
       <c r="G102" s="15"/>
-    </row>
-    <row r="103" spans="2:7">
+      <c r="H102" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="103" spans="2:8">
       <c r="B103" s="3" t="s">
         <v>100</v>
       </c>
@@ -3081,8 +3587,13 @@
       </c>
       <c r="F103" s="3"/>
       <c r="G103" s="15"/>
-    </row>
-    <row r="104" spans="2:7">
+      <c r="H103" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" spans="2:8">
       <c r="B104" s="3" t="s">
         <v>101</v>
       </c>
@@ -3097,8 +3608,13 @@
       </c>
       <c r="F104" s="3"/>
       <c r="G104" s="15"/>
-    </row>
-    <row r="105" spans="2:7">
+      <c r="H104" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" spans="2:8">
       <c r="B105" s="3" t="s">
         <v>102</v>
       </c>
@@ -3113,8 +3629,13 @@
       </c>
       <c r="F105" s="3"/>
       <c r="G105" s="15"/>
-    </row>
-    <row r="106" spans="2:7">
+      <c r="H105" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" spans="2:8">
       <c r="B106" s="3" t="s">
         <v>103</v>
       </c>
@@ -3129,8 +3650,13 @@
       </c>
       <c r="F106" s="3"/>
       <c r="G106" s="15"/>
-    </row>
-    <row r="107" spans="2:7">
+      <c r="H106" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" spans="2:8">
       <c r="B107" s="3" t="s">
         <v>104</v>
       </c>
@@ -3145,8 +3671,13 @@
       </c>
       <c r="F107" s="3"/>
       <c r="G107" s="15"/>
-    </row>
-    <row r="108" spans="2:7">
+      <c r="H107" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" spans="2:8">
       <c r="B108" s="3" t="s">
         <v>105</v>
       </c>
@@ -3161,8 +3692,13 @@
       </c>
       <c r="F108" s="3"/>
       <c r="G108" s="15"/>
-    </row>
-    <row r="109" spans="2:7">
+      <c r="H108" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" spans="2:8">
       <c r="B109" s="3" t="s">
         <v>106</v>
       </c>
@@ -3177,8 +3713,13 @@
       </c>
       <c r="F109" s="3"/>
       <c r="G109" s="15"/>
-    </row>
-    <row r="110" spans="2:7">
+      <c r="H109" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" spans="2:8">
       <c r="B110" s="3" t="s">
         <v>107</v>
       </c>
@@ -3193,8 +3734,13 @@
       </c>
       <c r="F110" s="3"/>
       <c r="G110" s="15"/>
-    </row>
-    <row r="111" spans="2:7" ht="33">
+      <c r="H110" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" spans="2:8" ht="33">
       <c r="B111" s="3" t="s">
         <v>108</v>
       </c>
@@ -3209,8 +3755,13 @@
       </c>
       <c r="F111" s="3"/>
       <c r="G111" s="15"/>
-    </row>
-    <row r="112" spans="2:7">
+      <c r="H111" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="112" spans="2:8">
       <c r="B112" s="3" t="s">
         <v>109</v>
       </c>
@@ -3225,8 +3776,13 @@
       </c>
       <c r="F112" s="3"/>
       <c r="G112" s="15"/>
-    </row>
-    <row r="113" spans="2:7">
+      <c r="H112" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="113" spans="2:8">
       <c r="B113" s="3" t="s">
         <v>110</v>
       </c>
@@ -3241,8 +3797,13 @@
       </c>
       <c r="F113" s="3"/>
       <c r="G113" s="15"/>
-    </row>
-    <row r="114" spans="2:7">
+      <c r="H113" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="114" spans="2:8">
       <c r="B114" s="3" t="s">
         <v>111</v>
       </c>
@@ -3257,8 +3818,13 @@
       </c>
       <c r="F114" s="3"/>
       <c r="G114" s="15"/>
-    </row>
-    <row r="115" spans="2:7">
+      <c r="H114" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="115" spans="2:8">
       <c r="B115" s="3" t="s">
         <v>112</v>
       </c>
@@ -3273,8 +3839,13 @@
       </c>
       <c r="F115" s="3"/>
       <c r="G115" s="15"/>
-    </row>
-    <row r="116" spans="2:7">
+      <c r="H115" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="116" spans="2:8">
       <c r="B116" s="3" t="s">
         <v>113</v>
       </c>
@@ -3289,8 +3860,13 @@
       </c>
       <c r="F116" s="3"/>
       <c r="G116" s="15"/>
-    </row>
-    <row r="117" spans="2:7" ht="33">
+      <c r="H116" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="117" spans="2:8" ht="33">
       <c r="B117" s="3" t="s">
         <v>114</v>
       </c>
@@ -3305,8 +3881,13 @@
       </c>
       <c r="F117" s="3"/>
       <c r="G117" s="15"/>
-    </row>
-    <row r="118" spans="2:7" ht="33">
+      <c r="H117" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="118" spans="2:8" ht="33">
       <c r="B118" s="3" t="s">
         <v>115</v>
       </c>
@@ -3321,8 +3902,13 @@
       </c>
       <c r="F118" s="3"/>
       <c r="G118" s="15"/>
-    </row>
-    <row r="119" spans="2:7" ht="33">
+      <c r="H118" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="119" spans="2:8" ht="33">
       <c r="B119" s="3" t="s">
         <v>116</v>
       </c>
@@ -3337,8 +3923,13 @@
       </c>
       <c r="F119" s="3"/>
       <c r="G119" s="15"/>
-    </row>
-    <row r="120" spans="2:7" ht="33">
+      <c r="H119" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="120" spans="2:8" ht="33">
       <c r="B120" s="3" t="s">
         <v>117</v>
       </c>
@@ -3353,8 +3944,13 @@
       </c>
       <c r="F120" s="3"/>
       <c r="G120" s="15"/>
-    </row>
-    <row r="121" spans="2:7" ht="33">
+      <c r="H120" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="121" spans="2:8" ht="33">
       <c r="B121" s="3" t="s">
         <v>118</v>
       </c>
@@ -3369,8 +3965,13 @@
       </c>
       <c r="F121" s="3"/>
       <c r="G121" s="15"/>
-    </row>
-    <row r="122" spans="2:7" ht="33">
+      <c r="H121" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="122" spans="2:8" ht="33">
       <c r="B122" s="3" t="s">
         <v>119</v>
       </c>
@@ -3385,8 +3986,13 @@
       </c>
       <c r="F122" s="3"/>
       <c r="G122" s="15"/>
-    </row>
-    <row r="123" spans="2:7" ht="33">
+      <c r="H122" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="123" spans="2:8" ht="33">
       <c r="B123" s="3" t="s">
         <v>120</v>
       </c>
@@ -3401,8 +4007,13 @@
       </c>
       <c r="F123" s="3"/>
       <c r="G123" s="15"/>
-    </row>
-    <row r="124" spans="2:7" ht="33">
+      <c r="H123" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="124" spans="2:8" ht="33">
       <c r="B124" s="3" t="s">
         <v>121</v>
       </c>
@@ -3417,6 +4028,11 @@
       </c>
       <c r="F124" s="3"/>
       <c r="G124" s="15"/>
+      <c r="H124" s="3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
     </row>
     <row r="125" spans="2:7" ht="20.25">
       <c r="B125" s="21" t="s">
@@ -3987,11 +4603,52 @@
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="E127:E131"/>
-    <mergeCell ref="B1:G1"/>
+    <mergeCell ref="B1:H1"/>
     <mergeCell ref="B149:G149"/>
     <mergeCell ref="B125:G125"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
+  <dataValidations count="13">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Use" error="ON 또는 OFF를 선택하세요." promptTitle="Use" prompt="ON: HwInp/HwOutp에 생성, OFF: Unused에 생성" sqref="H3:H124">
+      <formula1>"ON,OFF"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Type" error="이 핀이 지원하는 기능 중에서 선택하세요." promptTitle="Multi-port" prompt="핀 기능을 선택하세요 (easyConfig와 일치시킬 것)" sqref="C22 C78 C90">
+      <formula1>"AnalogSignal,DigitalSignal,ResistanceMeasurementSignal"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Type" error="이 핀이 지원하는 기능 중에서 선택하세요." promptTitle="Multi-port" prompt="핀 기능을 선택하세요 (easyConfig와 일치시킬 것)" sqref="C23:C25">
+      <formula1>"Frequency,DigitalSignal,AnalogSignal,CurrentSignal,ResistanceMeasurementSignal"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Type" error="이 핀이 지원하는 기능 중에서 선택하세요." promptTitle="Multi-port" prompt="핀 기능을 선택하세요 (easyConfig와 일치시킬 것)" sqref="C36:C39">
+      <formula1>"AnalogSignal,DigitalSignal,CurrentSignal,ResistanceMeasurementSignal"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Type" error="이 핀이 지원하는 기능 중에서 선택하세요." promptTitle="Multi-port" prompt="핀 기능을 선택하세요 (easyConfig와 일치시킬 것)" sqref="C43">
+      <formula1>"DigitalSignal,AnalogSignal,CurrentSignal,Frequency"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Type" error="이 핀이 지원하는 기능 중에서 선택하세요." promptTitle="Multi-port" prompt="핀 기능을 선택하세요 (easyConfig와 일치시킬 것)" sqref="C75 C94 C104">
+      <formula1>"AnalogSignal,DigitalSignal,ResistanceMeasurementSignal,Frequency,SENTSignal"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Type" error="이 핀이 지원하는 기능 중에서 선택하세요." promptTitle="Multi-port" prompt="핀 기능을 선택하세요 (easyConfig와 일치시킬 것)" sqref="C79">
+      <formula1>"ResistanceMeasurementSignal,DigitalSignal,AnalogSignal"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Type" error="이 핀이 지원하는 기능 중에서 선택하세요." promptTitle="Multi-port" prompt="핀 기능을 선택하세요 (easyConfig와 일치시킬 것)" sqref="C82 C95 C101:C102">
+      <formula1>"Frequency,DigitalSignal,AnalogSignal,ResistanceMeasurementSignal,SENTSignal"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Type" error="이 핀이 지원하는 기능 중에서 선택하세요." promptTitle="Multi-port" prompt="핀 기능을 선택하세요 (easyConfig와 일치시킬 것)" sqref="C83 C96 C98 C105">
+      <formula1>"AnalogSignal,DigitalSignal,CurrentSignal,Frequency"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Type" error="이 핀이 지원하는 기능 중에서 선택하세요." promptTitle="Multi-port" prompt="핀 기능을 선택하세요 (easyConfig와 일치시킬 것)" sqref="C85:C89">
+      <formula1>"DigitalSignal,AnalogSignal,CurrentSignal,ResistanceMeasurementSignal"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Type" error="이 핀이 지원하는 기능 중에서 선택하세요." promptTitle="Multi-port" prompt="핀 기능을 선택하세요 (easyConfig와 일치시킬 것)" sqref="C91:C92 C108:C110">
+      <formula1>"ResistanceMeasurementSignal,DigitalSignal,AnalogSignal,CurrentSignal"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Type" error="이 핀이 지원하는 기능 중에서 선택하세요." promptTitle="Multi-port" prompt="핀 기능을 선택하세요 (easyConfig와 일치시킬 것)" sqref="C100 C103">
+      <formula1>"SENTSignal,DigitalSignal,AnalogSignal,ResistanceMeasurementSignal,Frequency"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Type" error="이 핀이 지원하는 기능 중에서 선택하세요." promptTitle="Multi-port" prompt="핀 기능을 선택하세요 (easyConfig와 일치시킬 것)" sqref="C107">
+      <formula1>"PWMSignal,DigitalSignal,AnalogSignal"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Align multi-port descriptions with datasheet; _VI index for current inputs
- RC40_Pinmap.xlsx: fix Description of A21-A24 (Digital, Voltage, Frequency,
  Resistance) and K30 (Digital, Voltage, Current, Frequency, DSM1/DST1) per
  RE 95208 p.13-14/17-20; dropdowns rebuilt (all 36 multi-port pins now match)
- CurrentSignal (HwInp/AnI) uses the _VI pin id: AnI_as[DevInp_K42_VI_D]
  (cfg.currentIndexSuffix, default '_VI'); guide annotation updated
</commit_message>
<xml_diff>
--- a/RC40_Pinmap.xlsx
+++ b/RC40_Pinmap.xlsx
@@ -1893,8 +1893,10 @@
       <c r="D22" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="E22" s="1" t="s">
-        <v>192</v>
+      <c r="E22" s="1" t="inlineStr">
+        <is>
+          <t>Digital, Voltage, Frequency, Resistance</t>
+        </is>
       </c>
       <c r="F22" s="3"/>
       <c r="G22" s="15"/>
@@ -1914,8 +1916,10 @@
       <c r="D23" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="E23" s="1" t="s">
-        <v>195</v>
+      <c r="E23" s="1" t="inlineStr">
+        <is>
+          <t>Digital, Voltage, Frequency, Resistance</t>
+        </is>
       </c>
       <c r="F23" s="3"/>
       <c r="G23" s="15"/>
@@ -1935,8 +1939,10 @@
       <c r="D24" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="E24" s="1" t="s">
-        <v>195</v>
+      <c r="E24" s="1" t="inlineStr">
+        <is>
+          <t>Digital, Voltage, Frequency, Resistance</t>
+        </is>
       </c>
       <c r="F24" s="3"/>
       <c r="G24" s="15"/>
@@ -1956,8 +1962,10 @@
       <c r="D25" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="E25" s="1" t="s">
-        <v>195</v>
+      <c r="E25" s="1" t="inlineStr">
+        <is>
+          <t>Digital, Voltage, Frequency, Resistance</t>
+        </is>
       </c>
       <c r="F25" s="3"/>
       <c r="G25" s="15"/>
@@ -3002,8 +3010,10 @@
       <c r="D75" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="E75" s="1" t="s">
-        <v>194</v>
+      <c r="E75" s="1" t="inlineStr">
+        <is>
+          <t>Digital, Voltage, Current, Frequency, DSM1/DST1</t>
+        </is>
       </c>
       <c r="F75" s="3"/>
       <c r="G75" s="15"/>
@@ -4608,15 +4618,15 @@
     <mergeCell ref="B125:G125"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
-  <dataValidations count="13">
+  <dataValidations count="14">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Use" error="ON 또는 OFF를 선택하세요." promptTitle="Use" prompt="ON: HwInp/HwOutp에 생성, OFF: Unused에 생성" sqref="H3:H124">
       <formula1>"ON,OFF"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Type" error="이 핀이 지원하는 기능 중에서 선택하세요." promptTitle="Multi-port" prompt="핀 기능을 선택하세요 (easyConfig와 일치시킬 것)" sqref="C22 C78 C90">
-      <formula1>"AnalogSignal,DigitalSignal,ResistanceMeasurementSignal"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Type" error="이 핀이 지원하는 기능 중에서 선택하세요." promptTitle="Multi-port" prompt="핀 기능을 선택하세요 (easyConfig와 일치시킬 것)" sqref="C22">
+      <formula1>"AnalogSignal,DigitalSignal,ResistanceMeasurementSignal,Frequency"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Type" error="이 핀이 지원하는 기능 중에서 선택하세요." promptTitle="Multi-port" prompt="핀 기능을 선택하세요 (easyConfig와 일치시킬 것)" sqref="C23:C25">
-      <formula1>"Frequency,DigitalSignal,AnalogSignal,CurrentSignal,ResistanceMeasurementSignal"</formula1>
+      <formula1>"Frequency,DigitalSignal,AnalogSignal,ResistanceMeasurementSignal"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Type" error="이 핀이 지원하는 기능 중에서 선택하세요." promptTitle="Multi-port" prompt="핀 기능을 선택하세요 (easyConfig와 일치시킬 것)" sqref="C36:C39">
       <formula1>"AnalogSignal,DigitalSignal,CurrentSignal,ResistanceMeasurementSignal"</formula1>
@@ -4624,8 +4634,11 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Type" error="이 핀이 지원하는 기능 중에서 선택하세요." promptTitle="Multi-port" prompt="핀 기능을 선택하세요 (easyConfig와 일치시킬 것)" sqref="C43">
       <formula1>"DigitalSignal,AnalogSignal,CurrentSignal,Frequency"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Type" error="이 핀이 지원하는 기능 중에서 선택하세요." promptTitle="Multi-port" prompt="핀 기능을 선택하세요 (easyConfig와 일치시킬 것)" sqref="C75 C94 C104">
-      <formula1>"AnalogSignal,DigitalSignal,ResistanceMeasurementSignal,Frequency,SENTSignal"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Type" error="이 핀이 지원하는 기능 중에서 선택하세요." promptTitle="Multi-port" prompt="핀 기능을 선택하세요 (easyConfig와 일치시킬 것)" sqref="C75 C83 C96 C98 C105">
+      <formula1>"AnalogSignal,DigitalSignal,CurrentSignal,Frequency"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Type" error="이 핀이 지원하는 기능 중에서 선택하세요." promptTitle="Multi-port" prompt="핀 기능을 선택하세요 (easyConfig와 일치시킬 것)" sqref="C78 C90">
+      <formula1>"AnalogSignal,DigitalSignal,ResistanceMeasurementSignal"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Type" error="이 핀이 지원하는 기능 중에서 선택하세요." promptTitle="Multi-port" prompt="핀 기능을 선택하세요 (easyConfig와 일치시킬 것)" sqref="C79">
       <formula1>"ResistanceMeasurementSignal,DigitalSignal,AnalogSignal"</formula1>
@@ -4633,14 +4646,14 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Type" error="이 핀이 지원하는 기능 중에서 선택하세요." promptTitle="Multi-port" prompt="핀 기능을 선택하세요 (easyConfig와 일치시킬 것)" sqref="C82 C95 C101:C102">
       <formula1>"Frequency,DigitalSignal,AnalogSignal,ResistanceMeasurementSignal,SENTSignal"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Type" error="이 핀이 지원하는 기능 중에서 선택하세요." promptTitle="Multi-port" prompt="핀 기능을 선택하세요 (easyConfig와 일치시킬 것)" sqref="C83 C96 C98 C105">
-      <formula1>"AnalogSignal,DigitalSignal,CurrentSignal,Frequency"</formula1>
-    </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Type" error="이 핀이 지원하는 기능 중에서 선택하세요." promptTitle="Multi-port" prompt="핀 기능을 선택하세요 (easyConfig와 일치시킬 것)" sqref="C85:C89">
       <formula1>"DigitalSignal,AnalogSignal,CurrentSignal,ResistanceMeasurementSignal"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Type" error="이 핀이 지원하는 기능 중에서 선택하세요." promptTitle="Multi-port" prompt="핀 기능을 선택하세요 (easyConfig와 일치시킬 것)" sqref="C91:C92 C108:C110">
       <formula1>"ResistanceMeasurementSignal,DigitalSignal,AnalogSignal,CurrentSignal"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Type" error="이 핀이 지원하는 기능 중에서 선택하세요." promptTitle="Multi-port" prompt="핀 기능을 선택하세요 (easyConfig와 일치시킬 것)" sqref="C94 C104">
+      <formula1>"AnalogSignal,DigitalSignal,ResistanceMeasurementSignal,Frequency,SENTSignal"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Type" error="이 핀이 지원하는 기능 중에서 선택하세요." promptTitle="Multi-port" prompt="핀 기능을 선택하세요 (easyConfig와 일치시킬 것)" sqref="C100 C103">
       <formula1>"SENTSignal,DigitalSignal,AnalogSignal,ResistanceMeasurementSignal,Frequency"</formula1>

</xml_diff>

<commit_message>
K10/K31/K34/K74-K78: Pull-Up_32V per datasheet (ports PD_ -> PU_)
Datasheet RE 95208 p.14/p.20: these 0-32 V discrete inputs have a 14.7 kOhm
pull-up to Ubat (plus 80.2 kOhm pull-down); only A13/A25-A27/A40-A42 are
pull-down only. Port prefix changes from PD_ to PU_ for the 8 pins.
</commit_message>
<xml_diff>
--- a/RC40_Pinmap.xlsx
+++ b/RC40_Pinmap.xlsx
@@ -2758,8 +2758,10 @@
       <c r="D63" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="E63" s="1" t="s">
-        <v>191</v>
+      <c r="E63" s="1" t="inlineStr">
+        <is>
+          <t>Pull-Up_32V</t>
+        </is>
       </c>
       <c r="F63" s="3"/>
       <c r="G63" s="15"/>
@@ -3052,8 +3054,10 @@
       <c r="D77" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="E77" s="1" t="s">
-        <v>191</v>
+      <c r="E77" s="1" t="inlineStr">
+        <is>
+          <t>Pull-Up_32V</t>
+        </is>
       </c>
       <c r="F77" s="3"/>
       <c r="G77" s="15"/>
@@ -3115,8 +3119,10 @@
       <c r="D80" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="E80" s="1" t="s">
-        <v>191</v>
+      <c r="E80" s="1" t="inlineStr">
+        <is>
+          <t>Pull-Up_32V</t>
+        </is>
       </c>
       <c r="F80" s="3"/>
       <c r="G80" s="15"/>
@@ -3781,8 +3787,10 @@
       <c r="D112" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="E112" s="1" t="s">
-        <v>191</v>
+      <c r="E112" s="1" t="inlineStr">
+        <is>
+          <t>Pull-Up_32V</t>
+        </is>
       </c>
       <c r="F112" s="3"/>
       <c r="G112" s="15"/>
@@ -3802,8 +3810,10 @@
       <c r="D113" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="E113" s="1" t="s">
-        <v>191</v>
+      <c r="E113" s="1" t="inlineStr">
+        <is>
+          <t>Pull-Up_32V</t>
+        </is>
       </c>
       <c r="F113" s="3"/>
       <c r="G113" s="15"/>
@@ -3823,8 +3833,10 @@
       <c r="D114" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="E114" s="1" t="s">
-        <v>191</v>
+      <c r="E114" s="1" t="inlineStr">
+        <is>
+          <t>Pull-Up_32V</t>
+        </is>
       </c>
       <c r="F114" s="3"/>
       <c r="G114" s="15"/>
@@ -3844,8 +3856,10 @@
       <c r="D115" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="E115" s="1" t="s">
-        <v>191</v>
+      <c r="E115" s="1" t="inlineStr">
+        <is>
+          <t>Pull-Up_32V</t>
+        </is>
       </c>
       <c r="F115" s="3"/>
       <c r="G115" s="15"/>
@@ -3865,8 +3879,10 @@
       <c r="D116" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="E116" s="1" t="s">
-        <v>191</v>
+      <c r="E116" s="1" t="inlineStr">
+        <is>
+          <t>Pull-Up_32V</t>
+        </is>
       </c>
       <c r="F116" s="3"/>
       <c r="G116" s="15"/>

</xml_diff>